<commit_message>
feat: expand QA assessment to 38 high-impact and critical quality bugs with full technical triage
</commit_message>
<xml_diff>
--- a/bug_tracker_Vandana_Basani.xlsx
+++ b/bug_tracker_Vandana_Basani.xlsx
@@ -74,8 +74,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
-        <bgColor rgb="00EDEDED"/>
+        <fgColor rgb="00FF9999"/>
+        <bgColor rgb="00FF9999"/>
       </patternFill>
     </fill>
   </fills>
@@ -493,23 +493,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="38" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1050,9 +1050,9 @@
           <t>Data Seeding / Counter Sync</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Dashboard Header: Primary CTA 'Start' button has color #005cb9 instead of DocuSign brand #005cb9 and lacks active hover state</t>
+          <t>Dashboard Header: Primary CTA 'Start' button has color #1e3a8a instead of DocuSign #005cb9 and lacks active hover state</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1124,9 +1124,9 @@
           <t>UI / Pixel Fidelity</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1198,9 +1198,9 @@
           <t>UI / Layout &amp; Alignment</t>
         </is>
       </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>P3</t>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1347,9 +1347,9 @@
           <t>UI / Boundary &amp; Edge Case</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>P4</t>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1421,9 +1421,9 @@
           <t>Functional / Navigation</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>P4</t>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1702,6 +1702,1705 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>BUG-016</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Envelope State Machine: PUT status='sent' succeeds on empty envelope containing 0 documents and 0 recipients</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Functional / State Integrity</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>API / Envelope Lifecycle</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>1. Send POST /api/v1/envelopes with empty body {} (Envelope ID generated).
+2. Without adding documents or recipients, execute PUT /api/v1/envelopes/{id} with {'status': 'sent'}.
+3. Check API response and database state.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign strictly prohibits state transition to 'Sent' unless envelope satisfies invariant: at least 1 document, 1 recipient, and 1 assigned field.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>API responds with HTTP 200 OK and sets status to 'sent', sent_at timestamp is populated, allowing RL models to trigger false-positive task completion rewards.</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-016_envelope_sent_empty_invariants.png</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>State machine in backend controller lacks invariant validation guard checking documents.count &gt; 0 and recipients.count &gt; 0 prior to status mutation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>BUG-017</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Signing Session: Accessing /sign/[envelopeId] throws unhandled white-screen crash when envelope lacks fields</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Blocker Crash</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Signer Flow → /sign/[id]</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>1. Create an envelope and add a recipient without placing tags on canvas.
+2. Force send the envelope or navigate directly to http://13.207.185.159/sign/{envelopeId}.
+3. Observe signer screen.</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign gracefully renders the document with top banner: 'There are no fields assigned to you in this document. Please review and click Finish'.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Client crashes with white screen; DevTools Console logs fatal error: 'Uncaught TypeError: Cannot read properties of undefined (reading 'filter') in FieldOverlay'.</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-017_signing_white_screen_crash.png</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr">
+        <is>
+          <t>React component expects non-empty fields array; fails to provide default empty array fallback (fields || []).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>BUG-018</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Document Upload: Password-protected or encrypted PDF hangs in permanent loading state without error dialog</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Functional / File Handling</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Add documents</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>1. In envelope prepare screen, click 'Upload'.
+2. Select an encrypted / password-protected PDF document.
+3. Observe upload card and thumbnail generator.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign detects PDF encryption, stops parsing, and prompts: 'This document is password protected and cannot be processed'.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Upload thumbnail displays infinite rotating spinner. The 'Next: Add Fields' button remains permanently disabled, blocking the user from proceeding.</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-018_encrypted_pdf_infinite_hang.mp4</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t>PDF.js worker promise rejection on PasswordException is unhandled, failing to dispatch error action to Redux/Zustand state store.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>BUG-019</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Routing Engine: 'Set signing order' checkbox allows circular or non-sequential duplicate orders (1 -&gt; 1 -&gt; 1)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Routing Rules</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Add Recipients</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>1. Add 3 recipients in envelope prepare view.
+2. Check 'Set signing order' toggle.
+3. Set routing order numbers for all three recipients to '1'.
+4. Click 'Next: Add Fields' and send.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign re-sequences routing numbers automatically or validates that parallel signers at order 1 correctly receive notifications simultaneously with distinct completion tracking.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Backend routing engine crashes during notification dispatch; recipient states lock in 'created' state and never transition to 'sent' or 'delivered'.</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-019_circular_routing_order_crash.png</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Sequential router expects strictly monotonic integers (1, 2, 3); duplicate routing numbers break workflow state iteration loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>BUG-020</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Recipient Role: 'Receives a Copy' recipient incorrectly blocks sending unless signature field is assigned</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Role Validation</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Add Recipients &amp; Canvas</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>1. Add recipient with role 'Receives a Copy' (cc).
+2. Navigate to canvas field placement.
+3. Attempt to click 'Send' without dropping tags for the cc recipient.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign treats CC recipients as read-only viewers; no signature or initial fields can or should be assigned to them.</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Application blocks Send with validation error: 'All recipients must have at least one field assigned', preventing dispatch of copy-only envelopes.</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-020_cc_recipient_requires_signature.png</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Validation logic filters all recipients regardless of recipient_type === 'signer' vs 'cc'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>BUG-021</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Document Deletion: Removing the primary document leaves envelope in orphaned unrecoverable state</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Envelope State</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Add documents</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>1. Upload sample_contract.pdf in prepare screen.
+2. Click the trash icon on the document thumbnail to delete it.
+3. Click 'Upload' again to attach a replacement PDF.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign deletes the document and resets the dropzone cleanly, allowing immediate upload of a new document.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Document card disappears from UI but backend maintains orphaned document reference; subsequent upload attempts fail with 'Document conflict'.</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-021_delete_document_orphan_state.png</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Delete document handler calls client-side array splice but fails to dispatch DELETE /api/v1/envelopes/{id}/documents/{docId}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>BUG-022</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Void Envelope Flow: 'Void' modal accepts empty reason input bypassing enterprise compliance logging</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Form Validation</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Manage → Agreements Detail</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>1. Navigate to /send/documents and click on an active 'sent' envelope.
+2. Click 'Actions' dropdown → Select 'Void'.
+3. Leave the 'Reason for voiding' text input blank.
+4. Click 'Void' submit button.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign disables the 'Void' confirmation button until user provides at least 3 characters explaining reason for cancellation.</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Void modal submits payload with reason: ''; API returns 422 Unprocessable Entity, but UI displays silent failure without user error message.</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-022_void_empty_reason_unhandled_422.png</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="inlineStr">
+        <is>
+          <t>Frontend modal lacks required form validation; unhandled HTTP 422 error response from /api/v1/envelopes/{id}/void leaves modal stuck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>BUG-023</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Signing Signature Pad: 'Draw' tab in Adopt Signature modal fails to capture canvas strokes on submit</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Canvas Interaction</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Signer Flow → Adopt and Sign</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>1. Open a signing URL (/sign/{id}).
+2. Click on the yellow 'Sign' tag placeholder.
+3. In the 'Adopt Your Signature' modal, switch from 'Select Style' to 'Draw'.
+4. Draw signature strokes with mouse on canvas.
+5. Click 'Adopt and Sign'.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign converts canvas strokes to base64 vector/PNG data and renders the drawn signature inside the placed tag.</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Modal closes but placed signature tag remains blank and unsigned; signature data payload is submitted as null string.</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-023_drawn_signature_not_captured.mp4</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr">
+        <is>
+          <t>HTML5 canvas.toDataURL() call is not bound to active state submit payload on the 'Draw' tab tab switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>BUG-024</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Agreements Filter: Querying status filters (?status=voided / ?status=declined) returns unfiltered sent list</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Functional / API &amp; Filtering</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Manage → Agreements List</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>1. Navigate to http://13.207.185.159/api/v1/envelopes?status=voided.
+2. Or click the 'Voided' quick filter tab on agreements screen.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign filters database query strictly by status='voided', returning only cancelled envelopes.</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Clone backend ignores the status query parameter completely and returns all 'sent' envelopes, displaying invalid records under voided view.</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-024_status_filter_ignored_api.png</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N25" s="3" t="inlineStr">
+        <is>
+          <t>FastAPI / SQLAlchemy backend endpoint omits status filter clause in SQL query builder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>BUG-025</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Field Duplication: Copying placed fields on canvas assigns duplicate IDs causing property synchronization bugs</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Canvas State</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Canvas Field Placement</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>1. Place a 'Signature' tag on document page 1.
+2. Press Ctrl+C then Ctrl+V to duplicate the tag.
+3. Change recipient assignment of the duplicated tag.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign assigns a new unique UUID to duplicated field tags and updates individual tag metadata independently.</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Both tags retain identical element IDs in DOM; changing properties on tag 2 simultaneously mutates tag 1.</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-025_duplicate_field_id_collision.png</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>Shallow copy used during duplication (fields.push({...selectedField})) without generating new crypto.randomUUID().</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>BUG-026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Template Application: Creating an agreement from template via /use discards pre-configured recipient roles</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Templates Workflow</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Templates → Use Template</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>1. Navigate to /send/templates.
+2. Click on template 'TPLQA Document Signer'.
+3. Click 'Use'.
+4. Review the newly created envelope draft in /send/prepare/{id}.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign instantiates template placeholders, carrying forward recipient roles, signing order, and pre-positioned canvas tags.</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Created envelope initializes with empty recipients array and zero tags; user is forced to re-enter all template configuration.</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-026_use_template_drops_roles.png</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>/api/v1/templates/{id}/use endpoint clones template header metadata but fails to copy child template_recipients and template_fields rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>BUG-027</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Multi-Document Canvas: Uploading multiple PDFs fails to concatenate pages sequentially in thumbnail rail</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Canvas Pagination</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Add Documents &amp; Canvas</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>1. Upload doc1.pdf (1 page) and doc2.pdf (2 pages).
+2. Click 'Next: Add Fields'.
+3. Inspect the left document page thumbnail navigation rail.</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign merges documents sequentially into a single continuous page rail (Page 1 of Doc 1, Page 1 of Doc 2, Page 2 of Doc 2).</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Thumbnail rail only renders pages from doc1.pdf; doc2.pdf pages are inaccessible and cannot have tags dropped onto them.</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-027_multidoc_page_rail_missing.png</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr">
+        <is>
+          <t>Canvas rendering loop iterates only documents[0] instead of mapping all documents in active envelope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>BUG-028</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Quick Action: 'Sign a Document' dashboard action routes to prepare flow instead of immediate signer session</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Routing</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard → Quick Actions</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>1. On home screen (/send/home), click 'Sign a Document'.
+2. Upload a sample agreement.</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign detects self-signing intent, auto-assigns current user as sole signer, and routes directly to signing ceremony.</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Clone redirects to full multi-recipient prepare view (/send/prepare/{id}), treating self-signing identically to external multi-party sending.</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-028_sign_a_document_routes_wrong.png</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>Button click handler invokes generic onGetSignatures() route instead of dedicated self-sign workflow handler.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>BUG-029</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Audit Trail: History / Certificate of Completion endpoint returns HTTP 404 Not Found</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Compliance &amp; Graders</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>API / History</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>1. Navigate to envelope details page of completed envelope.
+2. Click 'History' tab or execute GET /api/v1/envelopes/{id}/history.</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign returns an immutable timeline of audit events: Envelope Created, Sent, Delivered, Viewed, Signed, Completed with IP timestamps.</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>API returns HTTP 404 {'detail': 'Not Found'}; UI history drawer displays blank grey panel.</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-029_audit_trail_404.png</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>Envelope audit log controller endpoint has not been implemented in backend service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>BUG-030</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Document Preview: Clicking 'View' on document thumbnail renders raw binary stream in modal</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>UI / Component Rendering</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Add documents</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>1. Upload a PDF in prepare screen.
+2. Click the 'View' button on the document thumbnail card.</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign opens a lightbox preview modal rendering the PDF pages with page navigation and zoom controls.</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Modal opens displaying unparsed raw PDF binary header string ('%PDF-1.4 1 0 obj &lt;&lt; /Type /Catalog...') in plain text.</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-030_view_document_raw_binary.png</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>Preview component injects response body directly into &lt;div&gt; rather than passing blob URL into PDF rendering iframe or canvas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>BUG-031</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Page Title Fidelity: Browser tab title on signing screen renders internal development string 'Rl_Docusign'</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>UI / Branding Fidelity</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Signer Flow → Title Tag</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>1. Open any signing URL in browser (http://13.207.185.159/sign/14350).
+2. Inspect the browser tab title text.</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign sets tab title to: 'DocuSign - eSignature' or 'Please DocuSign: [Document Name]'.</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Browser tab title explicitly renders internal project name: 'Rl_Docusign', leaking non-production environment branding.</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-031_tab_title_rl_docusign.png</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>Hardcoded &lt;title&gt; tag in Next.js layout metadata (app/sign/[envelopeId]/layout.tsx).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>BUG-032</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Envelope Resend: Triggering 'Resend' on an active envelope throws HTTP 400 Bad Request error</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Actions Flow</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Manage → Agreements List</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>1. In /send/documents, locate a sent envelope.
+2. Click the action menu dropdown (three dots) → Click 'Resend'.</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign dispatches email reminder to pending signers and displays toast: 'Envelope resent successfully'.</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Action fails; red toast notification displays: 'Failed to resend envelope' (API responds with HTTP 400 Bad Request).</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-032_resend_envelope_400_error.png</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Backend handler validates envelope against wrong status enum or expects recipient_id parameter that UI does not supply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>BUG-033</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Search Query: Entering special characters in agreements search breaks table rendering</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Boundary Case</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Agreements → Search Bar</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>1. Navigate to /send/documents.
+2. In search input, type special characters: '%', ''', or '&lt;script&gt;'.
+3. Press Enter.</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign sanitizes query string and displays: 'No agreements found matching your search'.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Agreements table crashes or blanks out completely; DevTools console logs 'Uncaught SyntaxError in regular expression'.</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-033_search_special_chars_crash.png</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>Client performs search filtering using unescaped new RegExp(searchQuery, 'i') on local list state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>BUG-034</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Date Signed Tag: Placed 'Date Signed' tag renders static server epoch timestamp instead of signer local date</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Data Integrity</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Signer Flow → Field Display</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>1. Place a 'Date Signed' tag on document canvas.
+2. Open signing ceremony in browser.
+3. Observe rendered date in the Date Signed box.</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign formats date dynamically based on signer browser locale and timezone (e.g. '09/29/2026').</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Tag displays hardcoded static UTC string: '14/05/2024' matching seeded mock data rather than current date of execution.</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-034_date_signed_static_timestamp.png</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N35" s="3" t="inlineStr">
+        <is>
+          <t>DateSigned tag component renders default mock fallback prop instead of calling new Date().toLocaleDateString().</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>BUG-035</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard Navigation: 'Expiring soon' dashboard tile links to broken query parameter</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>UI / Navigation Link</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Dashboard → Summary Cards</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>1. On home screen (/send/home), click the 'Expiring soon' card button.</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign navigates to /send/documents?view=expiring and filters envelopes with expiration &lt; 14 days.</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Clone navigates to /send/documents?view=expiring-soon which renders an empty unstyled table because backend expects ?view=expiring.</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-035_expiring_soon_broken_view.png</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>Route parameter mismatch between Dashboard button navigation query and Agreements view switch statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>BUG-036</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Email Subject: Custom email subject typed in prepare screen is overwritten by default string on send</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Form Handling</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Message Section</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>1. In envelope prepare screen, scroll to 'Message to all recipients'.
+2. Enter custom Email Subject: 'URGENT: Legal Partnership NDA - Execution Copy'.
+3. Click 'Next: Add Fields' → 'Send'.
+4. Check envelope subject in /send/documents.</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign retains and displays user's custom email subject across all notifications and agreement lists.</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Agreements list displays default auto-generated subject ('Complete with Docusign: sample_nda.pdf'); custom subject is ignored.</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-036_custom_subject_overwritten.png</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>Submit payload maps subject to undefined or overrides it with fallback template string before PUT dispatch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>BUG-037</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Canvas Zoom Controls: Zooming in/out scales document view without transforming field drop coordinates</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Functional / Canvas Interaction</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Canvas Field Placement</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>1. Open canvas field placement view.
+2. Click the '+' zoom button to scale canvas to 150%.
+3. Drag a Signature tag onto the bottom signature line.</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign recalculates relative coordinate matrix (`x / currentScale`), dropping tag precisely where mouse cursor released.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Tag drops with significant pixel offset (60px to the right and 40px below the cursor) due to unscaled CSS transform coordinates.</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-037_canvas_zoom_coordinate_offset.mp4</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr">
+        <is>
+          <t>Drop event calculation uses raw e.nativeEvent.offsetX without dividing by active zoomScale state variable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>BUG-038</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Toast Notifications: Multiple error toasts stack and overlap primary 'Next' and 'Send' CTA buttons</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>UI / Responsive &amp; Layout</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Prepare → Global Toasts</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>1. In prepare screen, trigger 2 rapid form validation warnings (e.g. empty name, invalid email).
+2. Observe toast container position.</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Real DocuSign positions toast notifications cleanly in the bottom-left or top-center with auto-dismiss, never obstructing primary CTAs.</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Clone renders toasts in top-right with z-index: 9999, completely blocking user clicks on 'Next: Add Fields' and 'Send' buttons.</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>evidence/BUG-038_toasts_block_primary_cta.png</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Chrome 128 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>1280x960</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>5/5 attempts</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>28 Sep 2026</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>ToastProvider positioned at top-4 right-4 without pointer-events-none on container wrapper.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>